<commit_message>
Bio Correction (Never Forget Way)
Changed the description of this location's memorial from 85th st to 84th st.
</commit_message>
<xml_diff>
--- a/data/total_edits.xlsx
+++ b/data/total_edits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/LLopez-Jensen/Documents/GitHub/9-11-memorials/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAA754D-457D-5242-8B08-FE92820AE1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{836BB2EF-17C4-1E4C-9BB3-3283B3988D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4089,9 +4089,6 @@
     <t>The Firemen’s Memorial in Riverside Park dates to 1913, and includes a grand staircase, a plaza, a fountain basin, and the central marble monument. It has long been a place of remembrance for firefighters who lost their lives in the line of duty, but after 9/11 it also became a place of gathering for vigils and annual remembrance ceremonies for the firefighters who were killed at the World Trade Center that day. Each year, a ceremony is held at the memorial with hundreds of U.S. flags arrayed around it honoring firefighters who were killed that day and the hundreds more that have died of 9/11 related illness since. </t>
   </si>
   <si>
-    <t>Along 85th Street, between 157th Ave and Shore Parkway in Queens, there are a number of 9/11 remembrances. A 9/11 tribute mural created by local artists and volunteers was unveiled in 2021 at a ‘Remembering September 11th’ ceremony below an overpass on the border between Howard Beach and Lindenwood. Howard Beach is home to many first responders, people who worked at Ground Zero in the months following the attacks and survivors of that tragic day. In 2022, just down the block, a Callery pear tree sapling from the original 9/11 survivor tree was planted in Howard Beach on the grounds of the former Rockwood Jewish Center. Annual remembrance events occur along this stretch, and within the nearby Our Lady of Grace, with very active community participation.   </t>
-  </si>
-  <si>
     <t>On September 11, 2001, the space at the corner of Beach Channel Drive and Beach 116th Street, facing Jamaica Bay, and thus the Twin Towers, was an undeveloped lot. The Rockaway Chamber of Commerce and the Friends of Tribute Park Committee worked to designate the space as a tribute park, which then occurred in 2005. The garden was designed by Lynden Miller and its pavilion by Patrick Clark. The park contains a mosaic centerpiece, a path of memorial bricks, and a granite rock with the engraved names of all 343 firefighters who lost their lives on September 11th. Annual remembrances, where 9/11 families place roses, have been held at the park.</t>
   </si>
   <si>
@@ -4204,6 +4201,9 @@
   </si>
   <si>
     <t>On American Veterans Memorial Pier, also known as the 69th Street Pier, is the September 11 Beacon memorial. It was designed and built by artist Robert Ressler, after being selected through a competition. The memorial, in the symbolic shape of a speaking trumpet once used by volunteer fire brigades, was cast from bronze at Bedi-Macky, a foundry in Greenpoint, and features a beacon of light shining from the top that is illuminated annually on September 11th. Annual vigils, often with performances by local school bands, such as nearby Xaverian High School, and ceremonials by scout troops, have been held on the pier, alongside the memorial.</t>
+  </si>
+  <si>
+    <t>Along 84th Street, between 157th Ave and Shore Parkway in Queens, there are a number of 9/11 remembrances. A 9/11 tribute mural created by local artists and volunteers was unveiled in 2021 at a ‘Remembering September 11th’ ceremony below an overpass on the border between Howard Beach and Lindenwood. Howard Beach is home to many first responders, people who worked at Ground Zero in the months following the attacks and survivors of that tragic day. In 2022, just down the block, a Callery pear tree sapling from the original 9/11 survivor tree was planted in Howard Beach on the grounds of the former Rockwood Jewish Center. Annual remembrance events occur along this stretch, and within the nearby Our Lady of Grace, with very active community participation.   </t>
   </si>
 </sst>
 </file>
@@ -4254,7 +4254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4263,7 +4263,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13776,7 +13775,7 @@
         <v>1212</v>
       </c>
       <c r="B327" t="s">
-        <v>1308</v>
+        <v>1332</v>
       </c>
       <c r="C327" t="s">
         <v>1213</v>
@@ -13811,7 +13810,7 @@
         <v>1214</v>
       </c>
       <c r="B328" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="C328" t="s">
         <v>1215</v>
@@ -13846,7 +13845,7 @@
         <v>1216</v>
       </c>
       <c r="B329" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="C329" t="s">
         <v>1217</v>
@@ -13881,7 +13880,7 @@
         <v>1219</v>
       </c>
       <c r="B330" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="C330" t="s">
         <v>1220</v>
@@ -13916,7 +13915,7 @@
         <v>1221</v>
       </c>
       <c r="B331" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C331" t="s">
         <v>1222</v>
@@ -13951,7 +13950,7 @@
         <v>1223</v>
       </c>
       <c r="B332" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="C332" t="s">
         <v>1224</v>
@@ -13986,7 +13985,7 @@
         <v>1225</v>
       </c>
       <c r="B333" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="C333" t="s">
         <v>1226</v>
@@ -14021,7 +14020,7 @@
         <v>1227</v>
       </c>
       <c r="B334" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="C334" t="s">
         <v>1228</v>
@@ -14056,7 +14055,7 @@
         <v>1230</v>
       </c>
       <c r="B335" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="C335" t="s">
         <v>1231</v>
@@ -14091,7 +14090,7 @@
         <v>1232</v>
       </c>
       <c r="B336" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="C336" t="s">
         <v>1233</v>
@@ -14126,7 +14125,7 @@
         <v>1235</v>
       </c>
       <c r="B337" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="C337" t="s">
         <v>1236</v>
@@ -14161,7 +14160,7 @@
         <v>1238</v>
       </c>
       <c r="B338" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="C338" t="s">
         <v>1239</v>
@@ -14196,7 +14195,7 @@
         <v>1243</v>
       </c>
       <c r="B339" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="C339" t="s">
         <v>1244</v>
@@ -14231,7 +14230,7 @@
         <v>1245</v>
       </c>
       <c r="B340" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C340" t="s">
         <v>1246</v>
@@ -14266,7 +14265,7 @@
         <v>1247</v>
       </c>
       <c r="B341" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C341" t="s">
         <v>1248</v>
@@ -14301,7 +14300,7 @@
         <v>1251</v>
       </c>
       <c r="B342" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="C342" t="s">
         <v>1252</v>
@@ -14336,7 +14335,7 @@
         <v>1254</v>
       </c>
       <c r="B343" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="C343" t="s">
         <v>1255</v>
@@ -14371,7 +14370,7 @@
         <v>1257</v>
       </c>
       <c r="B344" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="C344" t="s">
         <v>1258</v>
@@ -14406,7 +14405,7 @@
         <v>1260</v>
       </c>
       <c r="B345" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="C345" t="s">
         <v>1261</v>
@@ -14440,8 +14439,8 @@
       <c r="A346" t="s">
         <v>1264</v>
       </c>
-      <c r="B346" s="4" t="s">
-        <v>1327</v>
+      <c r="B346" t="s">
+        <v>1326</v>
       </c>
       <c r="C346" t="s">
         <v>1265</v>
@@ -14478,8 +14477,8 @@
       <c r="A347" t="s">
         <v>1267</v>
       </c>
-      <c r="B347" s="4" t="s">
-        <v>1328</v>
+      <c r="B347" t="s">
+        <v>1327</v>
       </c>
       <c r="C347" t="s">
         <v>1268</v>
@@ -14516,8 +14515,8 @@
       <c r="A348" t="s">
         <v>1269</v>
       </c>
-      <c r="B348" s="4" t="s">
-        <v>1329</v>
+      <c r="B348" t="s">
+        <v>1328</v>
       </c>
       <c r="C348" t="s">
         <v>1270</v>
@@ -14554,8 +14553,8 @@
       <c r="A349" t="s">
         <v>1274</v>
       </c>
-      <c r="B349" s="4" t="s">
-        <v>1330</v>
+      <c r="B349" t="s">
+        <v>1329</v>
       </c>
       <c r="C349" t="s">
         <v>1275</v>
@@ -14592,8 +14591,8 @@
       <c r="A350" t="s">
         <v>1276</v>
       </c>
-      <c r="B350" s="4" t="s">
-        <v>1331</v>
+      <c r="B350" t="s">
+        <v>1330</v>
       </c>
       <c r="C350" t="s">
         <v>1277</v>
@@ -14630,8 +14629,8 @@
       <c r="A351" t="s">
         <v>1278</v>
       </c>
-      <c r="B351" s="4" t="s">
-        <v>1332</v>
+      <c r="B351" t="s">
+        <v>1331</v>
       </c>
       <c r="C351" t="s">
         <v>1279</v>

</xml_diff>